<commit_message>
inspection update transpose, tambah amdal, inspection score < 60
</commit_message>
<xml_diff>
--- a/public/templates/template-ukl-upl.xlsx
+++ b/public/templates/template-ukl-upl.xlsx
@@ -15,6 +15,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="152511"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -24,10 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
-  <si>
-    <t>TEMPLATE MATRIKS UKL-UPL</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t>SUMBER DAMPAK</t>
   </si>
@@ -60,12 +58,6 @@
   </si>
   <si>
     <t>KETERANGAN</t>
-  </si>
-  <si>
-    <t>UPAYA PENGELOLAAN LINGKUNGAN HIDUP</t>
-  </si>
-  <si>
-    <t>UPAYA PEMANTAUAN LINGKUNGAN HIDUP</t>
   </si>
   <si>
     <t>(Tuliskan kegiatan yang menghasilkan dampak terhadap lingkungan)</t>
@@ -122,7 +114,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -145,15 +137,25 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -167,6 +169,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -447,188 +452,149 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="3" width="15" style="3" customWidth="1"/>
-    <col min="4" max="11" width="18.5703125" style="3" customWidth="1"/>
+    <col min="1" max="3" width="15" style="2" customWidth="1"/>
+    <col min="4" max="11" width="18.5703125" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:11" ht="75" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1"/>
-      <c r="C1"/>
-      <c r="D1"/>
-      <c r="E1"/>
-      <c r="F1"/>
-      <c r="G1"/>
-      <c r="H1"/>
-      <c r="I1"/>
-      <c r="J1"/>
-      <c r="K1"/>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="6" t="s">
+        <v>10</v>
+      </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="1"/>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1" t="s">
+    <row r="2" spans="1:11" ht="180" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1" t="s">
+      <c r="C2" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1"/>
-      <c r="J2" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>11</v>
+      <c r="D2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="60" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="J3" s="1"/>
-      <c r="K3" s="1"/>
+    <row r="3" spans="1:11" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="4"/>
+      <c r="B3" s="4"/>
+      <c r="C3" s="4"/>
+      <c r="D3" s="4"/>
+      <c r="E3" s="4"/>
+      <c r="F3" s="4"/>
+      <c r="G3" s="4"/>
+      <c r="H3" s="4"/>
+      <c r="I3" s="4"/>
+      <c r="J3" s="4"/>
+      <c r="K3" s="4"/>
     </row>
-    <row r="4" spans="1:11" ht="180" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="H4" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="I4" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="J4" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="K4" s="4" t="s">
-        <v>24</v>
-      </c>
+    <row r="4" spans="1:11" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="4"/>
+      <c r="B4" s="4"/>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4"/>
+      <c r="G4" s="4"/>
+      <c r="H4" s="4"/>
+      <c r="I4" s="4"/>
+      <c r="J4" s="4"/>
+      <c r="K4" s="4"/>
     </row>
-    <row r="5" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="5"/>
-      <c r="B5" s="5"/>
-      <c r="C5" s="5"/>
-      <c r="D5" s="5"/>
-      <c r="E5" s="5"/>
-      <c r="F5" s="5"/>
-      <c r="G5" s="5"/>
-      <c r="H5" s="5"/>
-      <c r="I5" s="5"/>
-      <c r="J5" s="5"/>
-      <c r="K5" s="5"/>
+    <row r="5" spans="1:11" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="4"/>
+      <c r="B5" s="4"/>
+      <c r="C5" s="4"/>
+      <c r="D5" s="4"/>
+      <c r="E5" s="4"/>
+      <c r="F5" s="4"/>
+      <c r="G5" s="4"/>
+      <c r="H5" s="4"/>
+      <c r="I5" s="4"/>
+      <c r="J5" s="4"/>
+      <c r="K5" s="4"/>
     </row>
-    <row r="6" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="5"/>
-      <c r="B6" s="5"/>
-      <c r="C6" s="5"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="5"/>
-      <c r="F6" s="5"/>
-      <c r="G6" s="5"/>
-      <c r="H6" s="5"/>
-      <c r="I6" s="5"/>
-      <c r="J6" s="5"/>
-      <c r="K6" s="5"/>
+    <row r="6" spans="1:11" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="4"/>
+      <c r="B6" s="4"/>
+      <c r="C6" s="4"/>
+      <c r="D6" s="4"/>
+      <c r="E6" s="4"/>
+      <c r="F6" s="4"/>
+      <c r="G6" s="4"/>
+      <c r="H6" s="4"/>
+      <c r="I6" s="4"/>
+      <c r="J6" s="4"/>
+      <c r="K6" s="4"/>
     </row>
-    <row r="7" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="5"/>
-      <c r="B7" s="5"/>
-      <c r="C7" s="5"/>
-      <c r="D7" s="5"/>
-      <c r="E7" s="5"/>
-      <c r="F7" s="5"/>
-      <c r="G7" s="5"/>
-      <c r="H7" s="5"/>
-      <c r="I7" s="5"/>
-      <c r="J7" s="5"/>
-      <c r="K7" s="5"/>
-    </row>
-    <row r="8" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="5"/>
-      <c r="B8" s="5"/>
-      <c r="C8" s="5"/>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
-      <c r="F8" s="5"/>
-      <c r="G8" s="5"/>
-      <c r="H8" s="5"/>
-      <c r="I8" s="5"/>
-      <c r="J8" s="5"/>
-      <c r="K8" s="5"/>
-    </row>
-    <row r="9" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="5"/>
-      <c r="B9" s="5"/>
-      <c r="C9" s="5"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
-      <c r="F9" s="5"/>
-      <c r="G9" s="5"/>
-      <c r="H9" s="5"/>
-      <c r="I9" s="5"/>
-      <c r="J9" s="5"/>
-      <c r="K9" s="5"/>
+    <row r="7" spans="1:11" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="4"/>
+      <c r="B7" s="4"/>
+      <c r="C7" s="4"/>
+      <c r="D7" s="4"/>
+      <c r="E7" s="4"/>
+      <c r="F7" s="4"/>
+      <c r="G7" s="4"/>
+      <c r="H7" s="4"/>
+      <c r="I7" s="4"/>
+      <c r="J7" s="4"/>
+      <c r="K7" s="4"/>
     </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="D2:F2"/>
-    <mergeCell ref="G2:I2"/>
-    <mergeCell ref="J2:J3"/>
-    <mergeCell ref="K2:K3"/>
-    <mergeCell ref="A2:C2"/>
-  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>